<commit_message>
chore: update Instagram report 2026-10-07 09:44
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/2026-10-07.xlsx
+++ b/instagram-daily-checker/reports/2026-10-07.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-10-07 09:11:43</t>
+          <t>取得日時：2026-10-07 09:44:15</t>
         </is>
       </c>
     </row>
@@ -736,12 +736,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+3人</t>
+          <t>+4人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">

</xml_diff>